<commit_message>
Deploy preview for PR 8 🛫
</commit_message>
<xml_diff>
--- a/pr-preview/pr-8/assets/coremeta4cat_vocabulary.xlsx
+++ b/pr-preview/pr-8/assets/coremeta4cat_vocabulary.xlsx
@@ -10542,7 +10542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J270"/>
+  <dimension ref="A1:J271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -21692,53 +21692,61 @@
       <c r="J264" s="12" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="12" t="inlineStr">
-        <is>
-          <t>column type</t>
-        </is>
-      </c>
-      <c r="B265" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C265" s="12" t="inlineStr">
+      <c r="A265" s="11" t="inlineStr">
+        <is>
+          <t>test slot 01</t>
+        </is>
+      </c>
+      <c r="B265" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C265" s="11" t="inlineStr">
         <is>
           <t>HighPerformanceLiquidChromatographyMassSpectrometry</t>
         </is>
       </c>
-      <c r="D265" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E265" s="12" t="inlineStr">
+      <c r="D265" s="11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E265" s="11" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F265" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G265" s="12" t="inlineStr"/>
-      <c r="H265" s="12" t="inlineStr"/>
-      <c r="I265" s="12" t="inlineStr">
-        <is>
-          <t>coremeta4cat:column_type</t>
-        </is>
-      </c>
-      <c r="J265" s="12" t="inlineStr">
-        <is>
-          <t>Type of chromatographic column used.</t>
+      <c r="F265" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G265" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H265" s="11" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="I265" s="11" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_slot_01</t>
+        </is>
+      </c>
+      <c r="J265" s="11" t="inlineStr">
+        <is>
+          <t>test_slot_01</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="12" t="inlineStr">
         <is>
-          <t>eluent</t>
+          <t>column type</t>
         </is>
       </c>
       <c r="B266" s="12" t="inlineStr">
@@ -21758,7 +21766,7 @@
       </c>
       <c r="E266" s="12" t="inlineStr">
         <is>
-          <t>ChemicalEntity</t>
+          <t>string</t>
         </is>
       </c>
       <c r="F266" s="12" t="inlineStr">
@@ -21766,27 +21774,23 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G266" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G266" s="12" t="inlineStr"/>
       <c r="H266" s="12" t="inlineStr"/>
       <c r="I266" s="12" t="inlineStr">
         <is>
-          <t>AFRL:0000011</t>
+          <t>coremeta4cat:column_type</t>
         </is>
       </c>
       <c r="J266" s="12" t="inlineStr">
         <is>
-          <t>Eluent or mobile phase used in chromatography.</t>
+          <t>Type of chromatographic column used.</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="12" t="inlineStr">
         <is>
-          <t>has flow rate</t>
+          <t>eluent</t>
         </is>
       </c>
       <c r="B267" s="12" t="inlineStr">
@@ -21806,27 +21810,35 @@
       </c>
       <c r="E267" s="12" t="inlineStr">
         <is>
-          <t>VolumeFlowRate</t>
-        </is>
-      </c>
-      <c r="F267" s="12" t="inlineStr"/>
-      <c r="G267" s="12" t="inlineStr"/>
+          <t>ChemicalEntity</t>
+        </is>
+      </c>
+      <c r="F267" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G267" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H267" s="12" t="inlineStr"/>
       <c r="I267" s="12" t="inlineStr">
         <is>
-          <t>SIO:000008</t>
+          <t>AFRL:0000011</t>
         </is>
       </c>
       <c r="J267" s="12" t="inlineStr">
         <is>
-          <t>Volumetric flow rate of a gas or liquid.</t>
+          <t>Eluent or mobile phase used in chromatography.</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="12" t="inlineStr">
         <is>
-          <t>has injection volume</t>
+          <t>has flow rate</t>
         </is>
       </c>
       <c r="B268" s="12" t="inlineStr">
@@ -21846,7 +21858,7 @@
       </c>
       <c r="E268" s="12" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>VolumeFlowRate</t>
         </is>
       </c>
       <c r="F268" s="12" t="inlineStr"/>
@@ -21859,14 +21871,14 @@
       </c>
       <c r="J268" s="12" t="inlineStr">
         <is>
-          <t>Volume injected in a chromatographic or mass spectrometric analysis.</t>
+          <t>Volumetric flow rate of a gas or liquid.</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="12" t="inlineStr">
         <is>
-          <t>external standard</t>
+          <t>has injection volume</t>
         </is>
       </c>
       <c r="B269" s="12" t="inlineStr">
@@ -21886,31 +21898,27 @@
       </c>
       <c r="E269" s="12" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F269" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="F269" s="12" t="inlineStr"/>
       <c r="G269" s="12" t="inlineStr"/>
       <c r="H269" s="12" t="inlineStr"/>
       <c r="I269" s="12" t="inlineStr">
         <is>
-          <t>coremeta4cat:external_standard</t>
+          <t>SIO:000008</t>
         </is>
       </c>
       <c r="J269" s="12" t="inlineStr">
         <is>
-          <t>External standard used for quantification or calibration.</t>
+          <t>Volume injected in a chromatographic or mass spectrometric analysis.</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="12" t="inlineStr">
         <is>
-          <t>internal standard</t>
+          <t>external standard</t>
         </is>
       </c>
       <c r="B270" s="12" t="inlineStr">
@@ -21942,10 +21950,54 @@
       <c r="H270" s="12" t="inlineStr"/>
       <c r="I270" s="12" t="inlineStr">
         <is>
+          <t>coremeta4cat:external_standard</t>
+        </is>
+      </c>
+      <c r="J270" s="12" t="inlineStr">
+        <is>
+          <t>External standard used for quantification or calibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="12" t="inlineStr">
+        <is>
+          <t>internal standard</t>
+        </is>
+      </c>
+      <c r="B271" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C271" s="12" t="inlineStr">
+        <is>
+          <t>HighPerformanceLiquidChromatographyMassSpectrometry</t>
+        </is>
+      </c>
+      <c r="D271" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E271" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F271" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G271" s="12" t="inlineStr"/>
+      <c r="H271" s="12" t="inlineStr"/>
+      <c r="I271" s="12" t="inlineStr">
+        <is>
           <t>coremeta4cat:internal_standard</t>
         </is>
       </c>
-      <c r="J270" s="12" t="inlineStr">
+      <c r="J271" s="12" t="inlineStr">
         <is>
           <t>Internal standard used for quantification or calibration.</t>
         </is>
@@ -21962,7 +22014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -22959,46 +23011,57 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>PlugFlowReactor</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>class</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>ChemicalReactor</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr"/>
-      <c r="F25" s="13" t="inlineStr"/>
-      <c r="G25" s="13" t="inlineStr"/>
-      <c r="H25" s="13" t="inlineStr"/>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>VOC4CAT:0007102</t>
-        </is>
-      </c>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>Plug flow reactor (PFR) — a tubular reactor in which reactant composition
-varies along the axis with no axial mixing.</t>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>testslot 5</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>CSTR</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr"/>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_uri_5</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>test_description_5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Autoclave</t>
+          <t>PlugFlowReactor</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -23022,20 +23085,20 @@
       <c r="H26" s="13" t="inlineStr"/>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>NCIT:C93052</t>
+          <t>VOC4CAT:0007102</t>
         </is>
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>Autoclave reactor — a sealed pressure vessel for batch reactions at
-elevated temperature and/or pressure.</t>
+          <t>Plug flow reactor (PFR) — a tubular reactor in which reactant composition
+varies along the axis with no axial mixing.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>SlurryReactor</t>
+          <t>Autoclave</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -23059,58 +23122,60 @@
       <c r="H27" s="13" t="inlineStr"/>
       <c r="I27" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:SlurryReactor</t>
+          <t>NCIT:C93052</t>
         </is>
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>Slurry reactor — a three-phase reactor in which catalyst particles are
-suspended in a liquid phase through which gas is bubbled.</t>
+          <t>Autoclave reactor — a sealed pressure vessel for batch reactions at
+elevated temperature and/or pressure.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>Microreactor</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>class</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>ChemicalReactor</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>testslot 4</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Autoclave</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr"/>
-      <c r="F28" s="13" t="inlineStr"/>
-      <c r="G28" s="13" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr"/>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>VOC4CAT:0000234</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>Microreactor — a miniaturised flow reactor with characteristic dimensions
-in the sub-millimetre range, enabling precise thermal control and rapid
-screening.</t>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr"/>
+      <c r="H28" s="11" t="inlineStr"/>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_uri_4</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>test_description_4</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>FixedBedReactor</t>
+          <t>SlurryReactor</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
@@ -23134,180 +23199,383 @@
       <c r="H29" s="13" t="inlineStr"/>
       <c r="I29" s="13" t="inlineStr">
         <is>
+          <t>coremeta4cat:SlurryReactor</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>Slurry reactor — a three-phase reactor in which catalyst particles are
+suspended in a liquid phase through which gas is bubbled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>testslot 3</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>SlurryReactor</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr"/>
+      <c r="G30" s="10" t="inlineStr"/>
+      <c r="H30" s="10" t="inlineStr"/>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_uri_3</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>test_description_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Microreactor</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>ChemicalReactor</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr"/>
+      <c r="F31" s="13" t="inlineStr"/>
+      <c r="G31" s="13" t="inlineStr"/>
+      <c r="H31" s="13" t="inlineStr"/>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>VOC4CAT:0000234</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>Microreactor — a miniaturised flow reactor with characteristic dimensions
+in the sub-millimetre range, enabling precise thermal control and rapid
+screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>testslot 1</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Microreactor</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr"/>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_uri_1</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>test_description_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>ChemicalReactor</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr"/>
+      <c r="F33" s="13" t="inlineStr"/>
+      <c r="G33" s="13" t="inlineStr"/>
+      <c r="H33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
           <t>coremeta4cat:FixedBedReactor</t>
         </is>
       </c>
-      <c r="J29" s="13" t="inlineStr">
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>Fixed bed reactor — a tubular reactor packed with a stationary catalyst bed.
 The most common reactor type in heterogeneous catalysis testing.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>testslot 2</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>FixedBedReactor</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr"/>
+      <c r="G34" s="12" t="inlineStr"/>
+      <c r="H34" s="12" t="inlineStr"/>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>VOC4CAT:test_uri_2</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>test_description_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>ChemicalReactor</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr"/>
-      <c r="F30" s="13" t="inlineStr"/>
-      <c r="G30" s="13" t="inlineStr"/>
-      <c r="H30" s="13" t="inlineStr"/>
-      <c r="I30" s="13" t="inlineStr">
+      <c r="E35" s="13" t="inlineStr"/>
+      <c r="F35" s="13" t="inlineStr"/>
+      <c r="G35" s="13" t="inlineStr"/>
+      <c r="H35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>coremeta4cat:FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="J30" s="13" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Fluidized bed reactor — a reactor in which the catalyst particles are
 suspended in an upward-flowing gas or liquid stream.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>gas distributor type</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="inlineStr"/>
-      <c r="H31" s="12" t="inlineStr"/>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr"/>
+      <c r="H36" s="12" t="inlineStr"/>
+      <c r="I36" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:gas_distributor_type</t>
         </is>
       </c>
-      <c r="J31" s="12" t="inlineStr">
+      <c r="J36" s="12" t="inlineStr">
         <is>
           <t>Type or design of the gas distributor plate in a fluidized bed reactor.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>bed expansion height</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="inlineStr"/>
-      <c r="H32" s="12" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr"/>
+      <c r="H37" s="12" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="I32" s="12" t="inlineStr">
+      <c r="I37" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bed_expansion_height</t>
         </is>
       </c>
-      <c r="J32" s="12" t="inlineStr">
+      <c r="J37" s="12" t="inlineStr">
         <is>
           <t>Height of bed expansion above the settled bed height under operating conditions.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>bubble size distribution</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>slot</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>slot</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
         <is>
           <t>FluidizedBedReactor</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr"/>
-      <c r="G33" s="12" t="inlineStr"/>
-      <c r="H33" s="12" t="inlineStr"/>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="F38" s="12" t="inlineStr"/>
+      <c r="G38" s="12" t="inlineStr"/>
+      <c r="H38" s="12" t="inlineStr"/>
+      <c r="I38" s="12" t="inlineStr">
         <is>
           <t>coremeta4cat:bubble_size_distribution</t>
         </is>
       </c>
-      <c r="J33" s="12" t="inlineStr">
+      <c r="J38" s="12" t="inlineStr">
         <is>
           <t>Description or characterization of bubble size distribution in the fluidized bed.</t>
         </is>

</xml_diff>